<commit_message>
Updating string parsing method
</commit_message>
<xml_diff>
--- a/data/cv.xlsx
+++ b/data/cv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\Private\git_laptop\curriculum-vitae\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D54006F-3615-4518-A397-67407188B741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F015A6-56C6-46CF-BD3C-BD1D8A49CB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21000" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="contact" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="223">
   <si>
     <t>position</t>
   </si>
@@ -108,9 +108,6 @@
   </si>
   <si>
     <t>activities</t>
-  </si>
-  <si>
-    <t>Present</t>
   </si>
   <si>
     <t>title</t>
@@ -323,9 +320,6 @@
     <t>mastodon</t>
   </si>
   <si>
-    <t>Doctoral researcher</t>
-  </si>
-  <si>
     <t>Zurich, Switzerland</t>
   </si>
   <si>
@@ -379,9 +373,6 @@
     <t>BSc with 1st Class Honours in Biological Sciences</t>
   </si>
   <si>
-    <t>ETH Zürich</t>
-  </si>
-  <si>
     <t>Edinburgh Napier University</t>
   </si>
   <si>
@@ -413,9 +404,6 @@
   </si>
   <si>
     <t>NAture-positive SCenarios for ENvironmental Transitions: Peru (NASCENT-PERU)</t>
-  </si>
-  <si>
-    <t>*Funded project under the SwissRE Biodiversity and Ecosystem Services Scenarios Modelling Initiative*</t>
   </si>
   <si>
     <t>Hungary, Greece, UK</t>
@@ -506,16 +494,6 @@
     <t>The Conservation Volunteers (TCV)</t>
   </si>
   <si>
-    <t>Produced protected area species inventories in line with Darwin Core standards utilising OpenRefine, R scripting and API services to expedite the collection of external data from the IUCN, EDGE ranking and CITES. Assisted in the training of new community biodiversity rangers in the process of SMART data collection in the field.</t>
-  </si>
-  <si>
-    <t>Coordinated safety and risk management as well as logistics for all centre activities including multi day field trips to remote locations in Cambodia and Vietnam. Medical ‘point person’, facilitated first aid training for staff. Performed pastoral role: ensuring student well-being, resolving group management issues and facilitating cultural adaptation.</t>
-  </si>
-  <si>
-    <t>Managed a diverse team (Bunong Indigenous minority, and Khmer) of 48 staff. Oversaw the operation of an ecotourism project receiving 4000+ visitors a year. Facilitated ongoing capacity building of staff and development of the volunteer program. 
-Compiled budgets, handled cash flow to staff and submitted detailed financial reports. Produced reports for the board of directors and Cambodian government. Developed relationships with other environmental and conservation organisations in the region.</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Planned, developed and delivered the Ochils Landscape Partnerships volunteering program and two TCV community health projects. Engaged with, and ensured the safety and wellbeing of a diverse cross section of volunteers, many with physical or mental disabilities as well as young adults/children.</t>
   </si>
   <si>
@@ -541,9 +519,6 @@
   </si>
   <si>
     <t>https://blenback.github.io/presentations/2021_06_09_ESP/</t>
-  </si>
-  <si>
-    <t>https://github.com/blenback/R-for-Reproducible-Research/</t>
   </si>
   <si>
     <t>https://plus.ethz.ch/research/forschungsprojekte/NASCENT-PERU.html/</t>
@@ -610,9 +585,6 @@
     <t>English</t>
   </si>
   <si>
-    <t>B1</t>
-  </si>
-  <si>
     <t>German</t>
   </si>
   <si>
@@ -622,9 +594,6 @@
     <t>Khmer</t>
   </si>
   <si>
-    <t>I am a PhD student currently working within the [**ValPar.CH**](https://valpar.ch/index_de.php) and [**NASCENT-Peru**](https://nascent-peru.github.io/) projects as part of the research group Planning of Landscape Urban Systems (PLUS) at ETH Zürich.</t>
-  </si>
-  <si>
     <t>Negotiating scenarios of a desirable ecological infrastructure for Switzerland</t>
   </si>
   <si>
@@ -650,6 +619,109 @@
   </si>
   <si>
     <t>https://blenback.github.io/presentations/2024_20_6_WBF/</t>
+  </si>
+  <si>
+    <t>Computational Urban Planning and Urban Management Conference 2025</t>
+  </si>
+  <si>
+    <t>University College London</t>
+  </si>
+  <si>
+    <t>Jun. 2025</t>
+  </si>
+  <si>
+    <t>https://virtual.oxfordabstracts.com/event/73503/submission/383</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>Nominated for the ETH medal for outstanding doctoral theses</t>
+  </si>
+  <si>
+    <t>A “Scope, Simulation and Story” approach to identify future spatial development scenarios</t>
+  </si>
+  <si>
+    <t>Post-Doctoral researcher</t>
+  </si>
+  <si>
+    <t>thesis</t>
+  </si>
+  <si>
+    <t>[Simulating the future potential of degraded Mangrove plots using field data from Kenya](http://dx.doi.org/10.13140/RG.2.2.20232.49923)</t>
+  </si>
+  <si>
+    <t>[Assessing the ecological effectiveness of protected areas in Cambodia: a quasi-experimental counterfactual estimation of avoided deforestation](http://dx.doi.org/10.13140/RG.2.2.28621.10727)</t>
+  </si>
+  <si>
+    <t>[Identifying effective area-based conservation strategies under uncertainties](https://blenback.github.io/presentations/2025_05_6_PhD_defence/)</t>
+  </si>
+  <si>
+    <t>https://blenback.github.io/R-for-Reproducible-Research/</t>
+  </si>
+  <si>
+    <t>I am a Post-Docotral researcher currently working within the [**ValPar.CH**](https://valpar.ch/index_de.php) and [**NASCENT-Peru**](https://nascent-peru.github.io/) projects as part of the research group Planning of Landscape Urban Systems (PLUS) at ETH Zürich. Active contributor to OMF and SwissRN</t>
+  </si>
+  <si>
+    <t>Funded project under the SwissRE Biodiversity and Ecosystem Services Scenarios Modelling Initiative</t>
+  </si>
+  <si>
+    <t>Dec. 2024</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>new</t>
+  </si>
+  <si>
+    <t>alt</t>
+  </si>
+  <si>
+    <t>test_alt</t>
+  </si>
+  <si>
+    <t>https://github.com/blenback/R-for-Reproducible-Research</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Developed a programmatic routine to expedite the collection of external data from the IUCN, EDGE ranking and CITES to produce protected area species inventories in line with Darwin Core standards. Assisted in the training of new community biodiversity rangers in the process of SMART data collection in the field.</t>
+  </si>
+  <si>
+    <t>Coordinated safety and risk management as well as logistics for all centre activities including multi day field trips to remote locations. Served as the medical point person, facilitating first aid training for staff, while also supporting student well-being and cultural adaptation in a pastoral role.</t>
+  </si>
+  <si>
+    <t>Managed a diverse team (Bunong Indigenous minority, and Khmer) of 48 staff. Oversaw the operation of an ecotourism project receiving 4000+ visitors a year. Facilitated ongoing capacity building of staff and development of the volunteer program. 
+Compiled budgets, managed cash flow, and created detailed financial and organizational reports.</t>
+  </si>
+  <si>
+    <t>Prognos AG</t>
+  </si>
+  <si>
+    <t>Jul. 2025</t>
+  </si>
+  <si>
+    <t>May. 2025</t>
+  </si>
+  <si>
+    <t>Freelance Research Consultant</t>
+  </si>
+  <si>
+    <t>Performed Land Use and Land Cover change modelling of Shared Socioeconomic Pathways for Switzerland as part of project funded by the Swiss National Centre for Climate Services</t>
+  </si>
+  <si>
+    <t>ETH Zürich, chair of Planning of Landscape Urban Systems (PLUS)</t>
+  </si>
+  <si>
+    <t>Feb. 2021</t>
+  </si>
+  <si>
+    <t>Jul. 2024</t>
+  </si>
+  <si>
+    <t>Participatory Environmental Modelling: MSc course at ETH Zürich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Designed and taught an MSc-level course integrating students and practitioners to develop simulation models for real-world environmental decision-making.  </t>
   </si>
 </sst>
 </file>
@@ -700,7 +772,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -710,6 +782,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1024,10 +1097,10 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
@@ -1039,45 +1112,45 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="F2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="G2" t="s">
         <v>93</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" t="s">
         <v>94</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>95</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>96</v>
       </c>
-      <c r="I2" t="s">
-        <v>97</v>
-      </c>
-      <c r="J2" t="s">
-        <v>98</v>
-      </c>
       <c r="M2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1091,7 +1164,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="54.7109375" customWidth="1"/>
@@ -1102,36 +1175,36 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
         <v>26</v>
-      </c>
-      <c r="E1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C2" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="D2" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1140,104 +1213,121 @@
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D3" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C5" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="D5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C6" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="C7" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="D7" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>180</v>
+      </c>
+      <c r="B8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" t="s">
         <v>190</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D9" t="s">
         <v>191</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E9" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="D8" t="s">
-        <v>141</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -1249,9 +1339,10 @@
     <hyperlink ref="E4" r:id="rId4" xr:uid="{A013CEAB-2FCD-4175-B64E-AFEFC4EBC399}"/>
     <hyperlink ref="E5" r:id="rId5" xr:uid="{F9DCC59D-DB81-4C87-A54D-F105942D3BD7}"/>
     <hyperlink ref="E8" r:id="rId6" xr:uid="{535CBEBE-B6BE-44AB-B4CE-F7D4B136C8B4}"/>
+    <hyperlink ref="E9" r:id="rId7" xr:uid="{36A93CC6-7FC4-4B20-8729-D9EFEA9C62D4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
 
@@ -1266,75 +1357,75 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
         <v>26</v>
-      </c>
-      <c r="E1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>57</v>
-      </c>
-      <c r="D2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" t="s">
         <v>53</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>54</v>
-      </c>
-      <c r="D3" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1354,27 +1445,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1382,7 +1473,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1393,13 +1484,13 @@
     </row>
     <row r="4" spans="1:4" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1407,13 +1498,13 @@
     </row>
     <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1421,13 +1512,13 @@
     </row>
     <row r="6" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6">
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -1453,26 +1544,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="B2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B3" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="B4" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -1502,7 +1593,7 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1510,7 +1601,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1518,7 +1609,7 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1526,7 +1617,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1534,7 +1625,7 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1542,7 +1633,7 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1550,7 +1641,7 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1600,67 +1691,79 @@
         <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>21</v>
+        <v>197</v>
       </c>
       <c r="G1" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" t="s">
         <v>108</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E2" t="s">
         <v>110</v>
       </c>
-      <c r="C2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E2" t="s">
-        <v>113</v>
+      <c r="F2" t="s">
+        <v>198</v>
       </c>
       <c r="G2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E3" t="s">
-        <v>115</v>
+        <v>112</v>
+      </c>
+      <c r="F3" t="s">
+        <v>199</v>
       </c>
       <c r="G3" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>218</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="D4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>191</v>
+      </c>
+      <c r="F4" t="s">
+        <v>200</v>
+      </c>
+      <c r="G4" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -1670,7 +1773,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
@@ -1703,102 +1806,122 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="E2" t="s">
-        <v>126</v>
-      </c>
-      <c r="F2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="E4" t="s">
         <v>128</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E3" t="s">
-        <v>132</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C4" t="s">
-        <v>135</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E4" t="s">
-        <v>137</v>
-      </c>
       <c r="F4" s="1" t="s">
-        <v>153</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" t="s">
-        <v>143</v>
+        <v>129</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>58</v>
+        <v>132</v>
       </c>
       <c r="E5" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>145</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6" t="s">
+        <v>140</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" t="s">
         <v>146</v>
       </c>
-      <c r="B6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E7" t="s">
+        <v>144</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="E6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1809,53 +1932,74 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="42.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="131" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="131" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
         <v>24</v>
-      </c>
-      <c r="B1" t="s">
-        <v>25</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
         <v>26</v>
       </c>
-      <c r="E1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D2" t="s">
-        <v>141</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>163</v>
+        <v>137</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B3" t="s">
+        <v>222</v>
+      </c>
+      <c r="C3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" t="s">
+        <v>219</v>
+      </c>
+      <c r="E3" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{08D31B25-1D87-4794-9C38-3A297CD026BD}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{08D31B25-1D87-4794-9C38-3A297CD026BD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1877,163 +2021,163 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>29</v>
       </c>
-      <c r="D1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>31</v>
-      </c>
-      <c r="G1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
         <v>42</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>43</v>
       </c>
-      <c r="C2" t="s">
-        <v>44</v>
-      </c>
       <c r="D2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s">
         <v>38</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>39</v>
       </c>
-      <c r="C3" t="s">
-        <v>40</v>
-      </c>
       <c r="D3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E4" t="s">
         <v>35</v>
-      </c>
-      <c r="D4" t="s">
-        <v>76</v>
-      </c>
-      <c r="E4" t="s">
-        <v>36</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" t="s">
         <v>70</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" t="s">
         <v>71</v>
-      </c>
-      <c r="C5" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" t="s">
-        <v>75</v>
-      </c>
-      <c r="E5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G5" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s">
         <v>77</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>78</v>
       </c>
-      <c r="C6" t="s">
-        <v>79</v>
-      </c>
       <c r="D6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F6" t="s">
         <v>9</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" t="s">
         <v>84</v>
       </c>
-      <c r="B7" t="s">
-        <v>85</v>
-      </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s">
         <v>9</v>
       </c>
       <c r="G7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2044,7 +2188,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
@@ -2055,7 +2199,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -2064,39 +2208,62 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
         <v>21</v>
       </c>
       <c r="F1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G1" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
+        <v>203</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="G2" t="s">
-        <v>89</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" t="s">
+        <v>206</v>
+      </c>
+      <c r="C3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E3" t="s">
+        <v>208</v>
+      </c>
+      <c r="F3" t="s">
+        <v>209</v>
+      </c>
+      <c r="G3" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update presentation section handling
</commit_message>
<xml_diff>
--- a/data/cv.xlsx
+++ b/data/cv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\Private\git_laptop\curriculum-vitae\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\git\curriculum-vitae\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BAC941-B287-4691-A407-1B1A128EB0A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2324F6CB-4F88-4408-86FE-3044BCFFDD88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="contact" sheetId="1" r:id="rId1"/>
@@ -2317,5 +2317,6 @@
     <hyperlink ref="F2" r:id="rId1" xr:uid="{A344B0D7-2544-4885-B67B-FC3F61A73CFD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
 </file>
</xml_diff>